<commit_message>
feat: reclassify Excel task outputs and restore candidates
</commit_message>
<xml_diff>
--- a/tasks/xlsx/cowork-bench-json-data-cleaning-pipeline/solution/Data_Pipeline_Report.xlsx
+++ b/tasks/xlsx/cowork-bench-json-data-cleaning-pipeline/solution/Data_Pipeline_Report.xlsx
@@ -10,11 +10,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales Analysis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Status" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined View" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Dashboard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sales Analysis'!$A$1:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inventory Status'!$A$1:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Combined View'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pipeline Dashboard'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Run Summary'!$A$1:$B$10</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -25,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="₽#,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,11 +41,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001F2937"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -75,19 +74,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -174,7 +170,7 @@
     <tableColumn id="3" name="Total_Revenue"/>
     <tableColumn id="4" name="Avg_Unit_Price"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -187,7 +183,7 @@
     <tableColumn id="3" name="Reorder_Point"/>
     <tableColumn id="4" name="Status"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -201,7 +197,32 @@
     <tableColumn id="4" name="Revenue"/>
     <tableColumn id="5" name="Stock_Status"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Pipeline_Dashboard" displayName="Pipeline_Dashboard" ref="A1:E6" headerRowCount="1">
+  <autoFilter ref="A1:E6"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Product_Name"/>
+    <tableColumn id="2" name="Total_Sold"/>
+    <tableColumn id="3" name="Current_Stock"/>
+    <tableColumn id="4" name="Revenue"/>
+    <tableColumn id="5" name="Stock_Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Pipeline_Run_Summary" displayName="Pipeline_Run_Summary" ref="A1:B10" headerRowCount="1">
+  <autoFilter ref="A1:B10"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Metric"/>
+    <tableColumn id="2" name="Value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -492,7 +513,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -503,7 +524,7 @@
     <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Product_Name</t>
@@ -525,99 +546,89 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Widget Alpha</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="3" t="n">
         <v>525</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="3" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Widget Beta</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="3" t="n">
         <v>850</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="3" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Gadget Pro</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="3" t="n">
         <v>850</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="3" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Sensor X1</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="3" t="n">
         <v>805</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Connector Z</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="3" t="n">
         <v>750</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="3" t="n">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D6"/>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;CCowork-Bench · Reproducible Data Cleaning</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -628,7 +639,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -639,7 +650,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Product_Name</t>
@@ -661,104 +672,94 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Widget Alpha</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <f>IF(B2&lt;=C2,"LOW","OK")</f>
         <v/>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Widget Beta</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f>IF(B3&lt;=C3,"LOW","OK")</f>
         <v/>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Gadget Pro</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f>IF(B4&lt;=C4,"LOW","OK")</f>
         <v/>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Sensor X1</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <f>IF(B5&lt;=C5,"LOW","OK")</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Connector Z</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <f>IF(B6&lt;=C6,"LOW","OK")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D6"/>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;CCowork-Bench · Reproducible Data Cleaning</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -769,7 +770,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -781,7 +782,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Product_Name</t>
@@ -808,106 +809,106 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Widget Alpha</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="3" t="n">
         <v>525</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Widget Beta</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="3" t="n">
         <v>850</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Gadget Pro</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="3" t="n">
         <v>850</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Sensor X1</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>805</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Connector Z</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="3" t="n">
         <v>750</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -915,17 +916,288 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E6"/>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;CCowork-Bench · Reproducible Data Cleaning</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Product_Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Sold</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Current_Stock</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Stock_Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Widget Alpha</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>525</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Widget Beta</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Gadget Pro</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Sensor X1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>805</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Connector Z</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>raw_sales_count</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>unique_sales_count</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>sales_duplicates_removed</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>raw_inventory_count</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>unique_inventory_count</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>inventory_duplicates_removed</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>total_quantity_sold</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>3780</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>low_stock_products</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>